<commit_message>
feature: InventoryManager에 hero 선택 기능, 초기 선택 기능 추가.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/GameErrorTable.xlsx
+++ b/input/Domains/Game/GameErrorTable.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1200" yWindow="500" windowWidth="37200" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GAME_ERROR" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="GAME_ERROR" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C189"/>
+  <dimension ref="A1:C193"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="59" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2686,6 +2686,54 @@
         </is>
       </c>
     </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>INVENTORY_HERO_LEVELUP_COUNT_INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Insufficient hero count to level up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>INVENTORY_CARD_LEVELUP_COUNT_INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Insufficient card count to level up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>INVENTORY_EQUIP_LEVELUP_MATERIAL_INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Insufficient level-up material to level up equip.</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>INVENTORY_ITEM_LEVELUP_CURRENCY_INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Insufficient currency to level up item.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>